<commit_message>
feat: verify rule CG0423 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000100/negative/01/data/unit-test-coreid-CG0423-negative.xlsx
+++ b/rules/CORE-000100/negative/01/data/unit-test-coreid-CG0423-negative.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -117,6 +123,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -560,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,6 +609,160 @@
         <is>
           <t>Error value</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AGTRT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Tuberculin PPD-S</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AGTRTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AGVAMT</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AGTRT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Tuberculin PPD-S</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AGTRTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AGVAMT</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -606,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -655,12 +825,12 @@
           <t>AGDOSU</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>AGTRTV</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>AGVAMT</t>
         </is>
@@ -672,63 +842,63 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>Reported Agent Name</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>AG Pre-Specified</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t>AG Occurrence</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>Dose per Administration</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>Dose Units</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="9" t="inlineStr">
         <is>
           <t>Treatment Vehicle</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>Treatment Vehicle
 Amount</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>Treatment Vehicle
 Amount Units</t>
@@ -736,102 +906,102 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="9" t="n">
         <v>50</v>
       </c>
     </row>
@@ -910,7 +1080,7 @@
       <c r="D6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Tuberculin PPD-S</t>
         </is>
@@ -933,11 +1103,63 @@
           <t>tuberculin unit</t>
         </is>
       </c>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="8" t="n">
+      <c r="J6" s="11" t="n"/>
+      <c r="K6" s="12" t="n">
         <v>0.1</v>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>mL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AG</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>XYZ-001-003</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Tuberculin PPD-S</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>tuberculin unit</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="n"/>
+      <c r="K7" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>mL</t>
         </is>

</xml_diff>